<commit_message>
Produce the 5 vertical social clips (V1-C1..V2-C3) per marketing plan
- marketing/clips/: five 9:16 1080x1920 clips cut from videos 1-2 with
  brand background, Arabic hook captions, salisauto.app footer, and the
  animated-logo outro with English VO audio kept from the source cuts
- gen_social.mjs: reusable generator for the vertical template assets
- Marketing plan + content calendar updated to mark clip assets ready

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017JYYQesysZ1mxqTEsUQv91
</commit_message>
<xml_diff>
--- a/video-series/marketing/content-calendar.xlsx
+++ b/video-series/marketing/content-calendar.xlsx
@@ -487,7 +487,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>المقاطع (V1-C1…V2-C3) مواصفات قصّها في MARKETING-PLAN-AR.md قسم ٣ — اطلب «جهّز مقاطع السوشال» لتوليدها من ملفات المستودع.</t>
+          <t>✅ المقاطع الخمسة (V1-C1…V2-C3) أُنتجت (٣ سبتمبر) وموجودة في marketing/clips/ — مواصفاتها في MARKETING-PLAN-AR.md قسم ٣.</t>
         </is>
       </c>
     </row>
@@ -630,7 +630,7 @@
       </c>
       <c r="F7" s="4" t="inlineStr">
         <is>
-          <t>V1-C1 (قص 0:26–0:46 من الفيديو ١، عمودي 9:16)</t>
+          <t>V1-C1 — ✅ جاهز: marketing/clips/salis-social-v1c1.mp4</t>
         </is>
       </c>
       <c r="G7" s="4" t="inlineStr">
@@ -704,7 +704,7 @@
       </c>
       <c r="F9" s="4" t="inlineStr">
         <is>
-          <t>V1-C2 (قص 0:08–0:24 من الفيديو ١، عمودي 9:16)</t>
+          <t>V1-C2 — ✅ جاهز: marketing/clips/salis-social-v1c2.mp4</t>
         </is>
       </c>
       <c r="G9" s="4" t="inlineStr">
@@ -741,7 +741,7 @@
       </c>
       <c r="F10" s="4" t="inlineStr">
         <is>
-          <t>V1-C1 (نفس مقطع تيك توك)</t>
+          <t>V1-C1 — ✅ جاهز: marketing/clips/salis-social-v1c1.mp4</t>
         </is>
       </c>
       <c r="G10" s="4" t="inlineStr">
@@ -889,7 +889,7 @@
       </c>
       <c r="F14" s="4" t="inlineStr">
         <is>
-          <t>V2-C1 (قص 0:14–0:36 من الفيديو ٢، عمودي 9:16)</t>
+          <t>V2-C1 — ✅ جاهز: marketing/clips/salis-social-v2c1.mp4</t>
         </is>
       </c>
       <c r="G14" s="4" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="F16" s="4" t="inlineStr">
         <is>
-          <t>V2-C2 (قص 0:46–1:06 من الفيديو ٢، عمودي 9:16)</t>
+          <t>V2-C2 — ✅ جاهز: marketing/clips/salis-social-v2c2.mp4</t>
         </is>
       </c>
       <c r="G16" s="4" t="inlineStr">
@@ -1000,7 +1000,7 @@
       </c>
       <c r="F17" s="4" t="inlineStr">
         <is>
-          <t>V2-C3 (قص 0:58–1:14 من الفيديو ٢)</t>
+          <t>V2-C3 — ✅ جاهز: marketing/clips/salis-social-v2c3.mp4</t>
         </is>
       </c>
       <c r="G17" s="4" t="inlineStr">

</xml_diff>

<commit_message>
Produce video 3 "customer journey" from the approved plan
- renders/video3-customer-journey.mp4: 80s, real recorded footage of the
  Arabic customer portal (quick login as Khalid, six-stage service journey
  for job A3F8B2C1, five vehicles, booking flow up to time selection,
  pending quote EST-0230, appointments and invoices), English VO with
  Saudi-dialect burned-in subtitles per the approved format
- record3.mjs / gen_caps3.mjs / tts3.py: video-3 pipeline scripts
- PLANNING-AR.md: video 3 marked produced
- Marketing plan + calendar: video-3 derivation (V3-C1..C3 clip specs,
  posts, discussion points) and a third scheduled week (Sep 20-24)

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017JYYQesysZ1mxqTEsUQv91
</commit_message>
<xml_diff>
--- a/video-series/marketing/content-calendar.xlsx
+++ b/video-series/marketing/content-calendar.xlsx
@@ -87,7 +87,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -99,6 +99,9 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -465,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -480,7 +483,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>تقويم المحتوى — أسبوعا الإطلاق (٦–١٧ سبتمبر ٢٠٢٦) · أيام النشر: الأحد–الخميس · الحالة: مجدول / منشور / مؤجل</t>
+          <t>تقويم المحتوى — ثلاثة أسابيع (٦–٢٤ سبتمبر ٢٠٢٦) · أيام النشر: الأحد–الخميس · الحالة: مجدول / منشور / مؤجل</t>
         </is>
       </c>
     </row>
@@ -1041,6 +1044,265 @@
         </is>
       </c>
       <c r="G18" s="4" t="inlineStr">
+        <is>
+          <t>مجدول</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>٢٠/٩</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>الأحد</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>X (تويتر)</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>بوست + فيديو</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>كم مكالمة «وين وصلت سيارتي؟» تجيك باليوم؟ عميلك عنده بوابة يشوف فيها رحلة سيارته خطوة بخطوة، ويحجز ويعتمد عرض السعر بنفسه. جرّبها بحساب خالد → salisauto.app #سالس_أوتو</t>
+        </is>
+      </c>
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>الفيديو ٣ كامل (video3-customer-journey.mp4)</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>مجدول</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>٢٠/٩</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>الأحد</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>لينكدإن</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>منشور + فيديو</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>Your customers don't want to call for updates — they want to see them. SALIS AUTO's customer portal: live service journey, self-booking, quote approval. #SalisAuto #GarageManagement</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>الفيديو ٣ كامل</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>مجدول</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>٢١/٩</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>الاثنين</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>تيك توك + ريلز</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>مقطع قصير</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>احجز صيانتك وأنت بالسرير 😴 — أربع خطوات بدون مكالمة</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>V3-C2 (قص 0:36–0:50 من الفيديو ٣، عمودي 9:16)</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>مجدول</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>٢٢/٩</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>الثلاثاء</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>X (تويتر)</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="inlineStr">
+        <is>
+          <t>نقطة نقاش</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>كعميل ورشة: وش أكثر شي يقهرك — إنك ما تعرف وين وصلت سيارتك، ولا فاتورة تنزل عليك فجأة؟ 👇</t>
+        </is>
+      </c>
+      <c r="F22" s="6" t="inlineStr">
+        <is>
+          <t>— (نص فقط)</t>
+        </is>
+      </c>
+      <c r="G22" s="6" t="inlineStr">
+        <is>
+          <t>مجدول</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>٢٣/٩</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>الأربعاء</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>يوتيوب شورتس</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>مقطع قصير</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>عميلك يتابع سيارته بنفسه | عنوان: Can your customers track their car repair live?</t>
+        </is>
+      </c>
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>V3-C1 (قص 0:14–0:34 من الفيديو ٣، عمودي 9:16)</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>مجدول</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t>٢٣/٩</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>الأربعاء</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>سناب شات</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="inlineStr">
+        <is>
+          <t>ستوري</t>
+        </is>
+      </c>
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>عرض السعر يوصلك — ما تحتاج تسأل</t>
+        </is>
+      </c>
+      <c r="F24" s="6" t="inlineStr">
+        <is>
+          <t>V3-C3 (قص 0:50–1:10 من الفيديو ٣)</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>مجدول</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t>٢٤/٩</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t>الخميس</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>X (تويتر)</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>نقطة نقاش</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>لو ورشتك تعطيك رابط تتابع منه سيارتك لحظة بلحظة، بتغيّر ورشتك عشانه؟</t>
+        </is>
+      </c>
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>— (نص فقط)</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
         <is>
           <t>مجدول</t>
         </is>

</xml_diff>

<commit_message>
Produce the V3 vertical social clips (V3-C1..C3)
- marketing/clips/: three 9:16 clips cut from video 3 with the shared
  brand template (hook captions, salisauto.app footer, logo outro)
- gen_social_v3.mjs: V3 hook-overlay generator
- Marketing plan + calendar updated to mark V3 clip assets ready

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017JYYQesysZ1mxqTEsUQv91
</commit_message>
<xml_diff>
--- a/video-series/marketing/content-calendar.xlsx
+++ b/video-series/marketing/content-calendar.xlsx
@@ -1151,7 +1151,7 @@
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>V3-C2 (قص 0:36–0:50 من الفيديو ٣، عمودي 9:16)</t>
+          <t>V3-C2 — ✅ جاهز: marketing/clips/salis-social-v3c2.mp4</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
@@ -1225,7 +1225,7 @@
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>V3-C1 (قص 0:14–0:34 من الفيديو ٣، عمودي 9:16)</t>
+          <t>V3-C1 — ✅ جاهز: marketing/clips/salis-social-v3c1.mp4</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
@@ -1262,7 +1262,7 @@
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>V3-C3 (قص 0:50–1:10 من الفيديو ٣)</t>
+          <t>V3-C3 — ✅ جاهز: marketing/clips/salis-social-v3c3.mp4</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">

</xml_diff>